<commit_message>
separated excel for experiments
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 4\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E4A333-34CB-4862-9BA3-50B51F4A2078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3015561D-5835-407B-A7AB-EF303EF8D50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="21">
   <si>
     <t>Exp#</t>
   </si>
@@ -88,12 +88,6 @@
   </si>
   <si>
     <t>python approach_residual_fingerprint_forgery.py --zip_file Dataset.zip --dataset_dir Dataset --out_dir submission_temp_residual_s45 --zip_out submission_residual_s45.zip --strength 4.5 --sigmas 1.0,2.0,4.0 --aggregation median</t>
-  </si>
-  <si>
-    <t>Frequency Bandpass Forgery</t>
-  </si>
-  <si>
-    <t>python approach_frequency_bandpass_forgery.py --zip_file Dataset.zip --dataset_dir Dataset --out_dir submissions/submission_freq_s4 --zip_out submission_freq_s4.zip --strength 4</t>
   </si>
 </sst>
 </file>
@@ -437,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -667,20 +661,6 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
-        <v>17</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
latest best score with residual with strength 4 sigma 4
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 4\tml2026-team_XLIII-assignment_4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3015561D-5835-407B-A7AB-EF303EF8D50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F0D52A-E558-4180-9613-E1429D4E20B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="24">
   <si>
     <t>Exp#</t>
   </si>
@@ -88,6 +88,15 @@
   </si>
   <si>
     <t>python approach_residual_fingerprint_forgery.py --zip_file Dataset.zip --dataset_dir Dataset --out_dir submission_temp_residual_s45 --zip_out submission_residual_s45.zip --strength 4.5 --sigmas 1.0,2.0,4.0 --aggregation median</t>
+  </si>
+  <si>
+    <t>python approach_residual_fingerprint_forgery.py --zip_file Dataset.zip --dataset_dir Dataset --out_dir submission_temp_residual_s4_sig1 --zip_out submission_residual_s4_sig1.zip --strength 4 --sigmas 1.0 --aggregation median</t>
+  </si>
+  <si>
+    <t>python approach_residual_fingerprint_forgery.py --zip_file Dataset.zip --dataset_dir Dataset --out_dir submission_temp_residual_s4_sig2 --zip_out submission_residual_s4_sig2.zip --strength 4 --sigmas 2.0 --aggregation median</t>
+  </si>
+  <si>
+    <t>python approach_residual_fingerprint_forgery.py --zip_file Dataset.zip --dataset_dir Dataset --out_dir submission_temp_residual_s4_sig4 --zip_out submission_residual_s4_sig4.zip --strength 4 --sigmas 4.0 --aggregation median</t>
   </si>
 </sst>
 </file>
@@ -431,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -632,6 +641,9 @@
       <c r="C14" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="D14" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
@@ -659,6 +671,48 @@
       </c>
       <c r="D16" s="3" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>17</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>18</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.37154199999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated score for w4, w6 patch
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 4\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CA2FD9-727A-4269-BDC0-8806B93E6B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06FCFD7F-ACAF-46AB-9085-C0CB7968B6A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="51">
   <si>
     <t>Exp#</t>
   </si>
@@ -172,6 +172,12 @@
   </si>
   <si>
     <t>submission_per_wm_consistency_v1</t>
+  </si>
+  <si>
+    <t>submission_patch_balanced</t>
+  </si>
+  <si>
+    <t>Patch wm4 wm6 artifacts</t>
   </si>
 </sst>
 </file>
@@ -221,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -234,6 +240,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -515,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -1126,8 +1135,22 @@
         <v>0.44159399999999999</v>
       </c>
     </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="3">
+        <v>44</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D44" s="3">
+        <v>0.44165500000000002</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
further exps for wm4 and 6
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 4\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79DB79A3-5EBA-4F91-B80B-B532D3A88462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F607D97-0C4B-48A1-8154-AFB372CB76C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="66">
   <si>
     <t>Exp#</t>
   </si>
@@ -208,6 +208,21 @@
   </si>
   <si>
     <t>WM 4 Edge s020 sides</t>
+  </si>
+  <si>
+    <t>wm4 Edge and wm6 Peak</t>
+  </si>
+  <si>
+    <t>python approach_patch_wm4_wm6_artifacts.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_per_wm_consistency_v1.zip --out_dir wm4_edge_wm6_peak --zip_out wm4_edge_wm6_peak.zip --profile wm4_edge_wm6_peak --print_psnr</t>
+  </si>
+  <si>
+    <t>python approach_patch_wm4_wm6_artifacts.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_per_wm_consistency_v1.zip --out_dir wm4_edge_wm6_peak_2 --zip_out wm4_edge_wm6_peak_2.zip --profile wm4_edge_wm6_peak_2 --print_psnr</t>
+  </si>
+  <si>
+    <t>python approach_patch_wm4_wm6_artifacts.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_per_wm_consistency_v1.zip --out_dir wm4_edge_wm6_peak_3 --zip_out wm4_edge_wm6_peak_3.zip --profile wm4_edge_wm6_peak_3 --print_psnr</t>
+  </si>
+  <si>
+    <t>python approach_patch_wm4_wm6_artifacts.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_per_wm_consistency_v1.zip --out_dir wm4_edge_wm6_peak_4 --zip_out wm4_edge_wm6_peak_4.zip --profile wm4_edge_wm6_peak_4 --print_psnr</t>
   </si>
 </sst>
 </file>
@@ -554,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -1263,6 +1278,62 @@
         <v>10</v>
       </c>
     </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="3">
+        <v>51</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="3">
+        <v>52</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="3">
+        <v>53</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="3">
+        <v>54</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
latest best score for WM2
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79DB79A3-5EBA-4F91-B80B-B532D3A88462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8819131C-077E-467D-825A-F22C1B9A5267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="89">
   <si>
     <t>Exp#</t>
   </si>
@@ -208,6 +208,90 @@
   </si>
   <si>
     <t>WM 4 Edge s020 sides</t>
+  </si>
+  <si>
+    <t>submission_wm4_edge_s025_sides</t>
+  </si>
+  <si>
+    <t>submission_wm4_edge_s035_bottomcorners</t>
+  </si>
+  <si>
+    <t>WM 4 Edge s025 sides</t>
+  </si>
+  <si>
+    <t>WM 4 Edge s035 bottomcorners</t>
+  </si>
+  <si>
+    <t>submission_wm4_edge_s035_sides</t>
+  </si>
+  <si>
+    <t>WM 4 Edge s035 sides</t>
+  </si>
+  <si>
+    <t>submission_wm4_edge_s015_sides</t>
+  </si>
+  <si>
+    <t>WM 4 Edge s015 sides</t>
+  </si>
+  <si>
+    <t>submission_wm1_global_revert_sig4</t>
+  </si>
+  <si>
+    <t>WM1 sig4 last best</t>
+  </si>
+  <si>
+    <t>submission_wm1_no_freq</t>
+  </si>
+  <si>
+    <t>submission_wm1_sig6_s35</t>
+  </si>
+  <si>
+    <t>submission_wm1_sig8</t>
+  </si>
+  <si>
+    <t>submission_wm1_freq_narrow</t>
+  </si>
+  <si>
+    <t>submission_wm2_global_revert_sig4</t>
+  </si>
+  <si>
+    <t>WM 2 global revert sig4</t>
+  </si>
+  <si>
+    <t>WM 1 No Frew</t>
+  </si>
+  <si>
+    <t>WM1 sig6 s35</t>
+  </si>
+  <si>
+    <t>WM1 sig8</t>
+  </si>
+  <si>
+    <t>WM1 freq narrow</t>
+  </si>
+  <si>
+    <t>WM2 no freq</t>
+  </si>
+  <si>
+    <t>submission_wm2_no_freq</t>
+  </si>
+  <si>
+    <t>submission_wm2_freq_narrow</t>
+  </si>
+  <si>
+    <t>WM2 freq narrow</t>
+  </si>
+  <si>
+    <t>submission_wm2_sig6_s35</t>
+  </si>
+  <si>
+    <t>submission_wm2_sig8</t>
+  </si>
+  <si>
+    <t>wm2 sig8</t>
+  </si>
+  <si>
+    <t>wm2 sig6 S35</t>
   </si>
 </sst>
 </file>
@@ -554,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -1263,6 +1347,202 @@
         <v>10</v>
       </c>
     </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" s="3">
+        <v>51</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="3">
+        <v>52</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="3">
+        <v>53</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="3">
+        <v>54</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="3">
+        <v>55</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="3">
+        <v>56</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="3">
+        <v>57</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="3">
+        <v>58</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="3">
+        <v>59</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="3">
+        <v>60</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D60" s="3">
+        <v>0.44519700000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="3">
+        <v>61</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="3">
+        <v>62</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="3">
+        <v>63</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="3">
+        <v>64</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
updated latest results with wm3 improvement
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8819131C-077E-467D-825A-F22C1B9A5267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB3B3AF-607F-4330-BE85-F75A1C5BF0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="97">
   <si>
     <t>Exp#</t>
   </si>
@@ -292,6 +292,30 @@
   </si>
   <si>
     <t>wm2 sig6 S35</t>
+  </si>
+  <si>
+    <t>submission_wm3_ms_tone</t>
+  </si>
+  <si>
+    <t>submission_wm3_luma_strong</t>
+  </si>
+  <si>
+    <t>submission_wm3_ms_balanced</t>
+  </si>
+  <si>
+    <t>submission_wm3_highfreq_plus</t>
+  </si>
+  <si>
+    <t>submission_wm3_vignette_focus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wm3 </t>
+  </si>
+  <si>
+    <t>submission_wm3_freq_narrow</t>
+  </si>
+  <si>
+    <t>submission_wm3_sig8</t>
   </si>
 </sst>
 </file>
@@ -638,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -1543,6 +1567,118 @@
         <v>10</v>
       </c>
     </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="3">
+        <v>65</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="3">
+        <v>66</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="3">
+        <v>67</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="3">
+        <v>68</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="3">
+        <v>69</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="3">
+        <v>70</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="3">
+        <v>71</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D71" s="3">
+        <v>0.44581100000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="3">
+        <v>72</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D72" s="3">
+        <v>0.44808900000000002</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
updated best with wm 8 tuning
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 4\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB3B3AF-607F-4330-BE85-F75A1C5BF0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62D8D0CB-75D0-41F1-8A27-4062EDC470DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="106">
   <si>
     <t>Exp#</t>
   </si>
@@ -316,6 +316,33 @@
   </si>
   <si>
     <t>submission_wm3_sig8</t>
+  </si>
+  <si>
+    <t>wm_5678</t>
+  </si>
+  <si>
+    <t>python approach_wm5678_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_wm3_sig8.zip --wm WM_8 --profile wm8_sig8 --out_dir submission_temp_wm8_sig8 --zip_out submission_wm8_sig8.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm8_sig8.zip</t>
+  </si>
+  <si>
+    <t>python approach_wm5678_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_wm3_sig8.zip --wm WM_8 --profile wm8_sig10 --out_dir submission_temp_wm8_sig10 --zip_out submission_wm8_sig10.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm8_sig10.zip</t>
+  </si>
+  <si>
+    <t>python approach_wm5678_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_wm8_sig10.zip --wm WM_5 --profile wm5_sig2 --out_dir submission_temp_wm5_sig2 --zip_out submission_wm5_sig2.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm5_sig2.zip</t>
+  </si>
+  <si>
+    <t>python approach_wm5678_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_wm8_sig10.zip --wm WM_5 --profile wm5_sig1_2 --out_dir submission_temp_wm5_sig1_2 --zip_out submission_wm5_sig1_2.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm5_sig1_2.zip</t>
   </si>
 </sst>
 </file>
@@ -365,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -381,6 +408,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -1567,7 +1600,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>65</v>
       </c>
@@ -1581,7 +1614,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>66</v>
       </c>
@@ -1595,7 +1628,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>67</v>
       </c>
@@ -1609,7 +1642,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>68</v>
       </c>
@@ -1623,7 +1656,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>69</v>
       </c>
@@ -1637,7 +1670,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>70</v>
       </c>
@@ -1651,7 +1684,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>71</v>
       </c>
@@ -1665,7 +1698,7 @@
         <v>0.44581100000000001</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>72</v>
       </c>
@@ -1677,6 +1710,68 @@
       </c>
       <c r="D72" s="3">
         <v>0.44808900000000002</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="3">
+        <v>73</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D73" s="3">
+        <v>0.44998199999999999</v>
+      </c>
+      <c r="E73" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="3">
+        <v>74</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D74" s="3">
+        <v>0.45707799999999998</v>
+      </c>
+      <c r="E74" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="3">
+        <v>75</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E75" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="3">
+        <v>76</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E76" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added latest best zip
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 4\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB5A395-AFE7-4F6A-87E6-76ED88DC6CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{990BB9EE-57D0-4A80-884C-F6AD07A570C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="110">
   <si>
     <t>Exp#</t>
   </si>
@@ -343,6 +343,18 @@
   </si>
   <si>
     <t>submission_wm5_sig1_2.zip</t>
+  </si>
+  <si>
+    <t>python approach_wm5678_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_wm8_sig10.zip --wm WM_8 --profile wm8_sig12 --out_dir submission_temp_wm8_sig12 --zip_out submission_wm8_sig12.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm8_sig12.zip</t>
+  </si>
+  <si>
+    <t>python approach_wm5678_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip submission_wm8_sig10.zip --wm WM_5 --profile wm5_sig8 --out_dir submission_temp_wm5_sig8 --zip_out submission_wm5_sig8.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm5_sig8.zip</t>
   </si>
 </sst>
 </file>
@@ -695,7 +707,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -1780,6 +1792,37 @@
         <v>105</v>
       </c>
     </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="3">
+        <v>77</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C77" t="s">
+        <v>106</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E77" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="3">
+        <v>78</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E78" t="s">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
latest score with wm3"
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 4\tml2026-team_XLIII-assignment_4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{990BB9EE-57D0-4A80-884C-F6AD07A570C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F577B606-B4BC-46D6-AB0E-139D8D5BD00B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="111">
   <si>
     <t>Exp#</t>
   </si>
@@ -355,6 +355,9 @@
   </si>
   <si>
     <t>submission_wm5_sig8.zip</t>
+  </si>
+  <si>
+    <t>python approach_wm3_only_conservative.py  --zip_file Dataset.zip  --dataset_dir Dataset --base_zip latest_best_result.zip  --profile wm3_sig10  --out_dir submission_temp_wm3_sig10_from_wm2  --zip_out submission_wm3_sig10_from_wm2.zip  --print_psnr</t>
   </si>
 </sst>
 </file>
@@ -707,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -1823,6 +1826,20 @@
         <v>109</v>
       </c>
     </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="3">
+        <v>79</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D79" s="3">
+        <v>0.45798800000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
updated best with wm7
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UdS\Summer 2026\courses\TML\assignments\Assignment 4\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F577B606-B4BC-46D6-AB0E-139D8D5BD00B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{952E8C4F-0D73-420D-A645-025F7916445A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="120">
   <si>
     <t>Exp#</t>
   </si>
@@ -358,6 +358,33 @@
   </si>
   <si>
     <t>python approach_wm3_only_conservative.py  --zip_file Dataset.zip  --dataset_dir Dataset --base_zip latest_best_result.zip  --profile wm3_sig10  --out_dir submission_temp_wm3_sig10_from_wm2  --zip_out submission_wm3_sig10_from_wm2.zip  --print_psnr</t>
+  </si>
+  <si>
+    <t>python approach_wm3_only_conservative.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip latest_best_result.zip --profile wm3_sig12 --out_dir submission_temp_wm3_sig12 --zip_out submission_wm3_sig12.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm3_sig12.zip</t>
+  </si>
+  <si>
+    <t>python approach_wm1_only_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip latest_best_result.zip --profile wm1_sig10 --out_dir submission_temp_wm1_sig10 --zip_out submission_wm1_sig10.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm1_sig10.zip</t>
+  </si>
+  <si>
+    <t>wm1</t>
+  </si>
+  <si>
+    <t>python approach_wm5678_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip latest_best_result.zip --wm WM_6 --profile wm6_sig8 --out_dir submission_temp_wm6_sig8 --zip_out submission_wm6_sig8.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm6_sig8.zip</t>
+  </si>
+  <si>
+    <t>python approach_wm5678_experiments.py --zip_file Dataset.zip --dataset_dir Dataset --base_zip latest_best_result.zip --wm WM_7 --profile wm7_sig8 --out_dir submission_temp_wm7_sig8 --zip_out submission_wm7_sig8.zip --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm7_sig8.zip</t>
   </si>
 </sst>
 </file>
@@ -710,7 +737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -1822,6 +1849,9 @@
       <c r="C78" s="7" t="s">
         <v>108</v>
       </c>
+      <c r="D78" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="E78" t="s">
         <v>109</v>
       </c>
@@ -1838,6 +1868,74 @@
       </c>
       <c r="D79" s="3">
         <v>0.45798800000000001</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="3">
+        <v>80</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E80" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="3">
+        <v>81</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E81" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="3">
+        <v>82</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E82" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="3">
+        <v>83</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C83" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D83" s="3">
+        <v>0.463287</v>
+      </c>
+      <c r="E83" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
latest best score with wm7 trustmark forgery 0.80
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1D891C-8F8B-42A4-81CD-6E8663197E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA3CD2D-0A75-4158-8A7D-BA0DF7179229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="170">
   <si>
     <t>Exp#</t>
   </si>
@@ -545,6 +545,15 @@
   --base_zip submission_wm1_wm2_real.zip \
   --out_dir temp_wm8_dwtdct --zip_out submission_wm1_wm2_wm8_real.zip \
   --wm WM_8 --method dwtDct --n_bits 24 --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm7_trustmark</t>
+  </si>
+  <si>
+    <t>approach_trustmark_forgery.py \
+  --dataset_dir Dataset --base_zip latest_best_results_070.zip \
+  --out_dir temp_wm7 --zip_out submission_wm7_trustmark.zip \
+  --variant Q --print_psnr</t>
   </si>
 </sst>
 </file>
@@ -600,7 +609,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -622,9 +631,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -906,7 +912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -2464,46 +2470,60 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>106</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C106" s="8" t="s">
+      <c r="C106" s="6" t="s">
         <v>162</v>
       </c>
       <c r="D106" s="3">
         <v>0.57699999999999996</v>
       </c>
     </row>
-    <row r="107" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>107</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="C107" s="8" t="s">
+      <c r="C107" s="6" t="s">
         <v>165</v>
       </c>
       <c r="D107" s="3">
         <v>0.70099999999999996</v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>108</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C108" s="8" t="s">
+      <c r="C108" s="6" t="s">
         <v>167</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A109" s="3">
+        <v>109</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D109" s="3">
+        <v>0.80372100000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final best score 0.90
</commit_message>
<xml_diff>
--- a/Experiments.xlsx
+++ b/Experiments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SEM 5\TML\Assignments\Watermarking\tml2026-team_XLIII-assignment_4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEA3CD2D-0A75-4158-8A7D-BA0DF7179229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F40E8DFD-A462-4DFD-9E50-5F0059AF7909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="172">
   <si>
     <t>Exp#</t>
   </si>
@@ -554,6 +554,15 @@
   --dataset_dir Dataset --base_zip latest_best_results_070.zip \
   --out_dir temp_wm7 --zip_out submission_wm7_trustmark.zip \
   --variant Q --print_psnr</t>
+  </si>
+  <si>
+    <t>submission_wm8_trustmark</t>
+  </si>
+  <si>
+    <t>venv_trustmark/Scripts/python.exe approach_trustmark_forgery.py \
+  --dataset_dir Dataset --base_zip latest_best_results_080.zip \
+  --wm WM_8 --variant P \
+  --out_dir temp_wm8 --zip_out submission_wm8_trustmark.zip --print_psnr</t>
   </si>
 </sst>
 </file>
@@ -912,7 +921,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
@@ -2526,6 +2535,20 @@
         <v>0.80372100000000002</v>
       </c>
     </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" s="3">
+        <v>110</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D110" s="3">
+        <v>0.90100000000000002</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>